<commit_message>
Dynamic detection of column
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,16 +427,164 @@
           <t>Archivo</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Importe_11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1001</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>factura_001.pdf</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>109,15 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>53,72 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>87,73 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>53,72 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>37,64 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>53,72 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>85,91 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>53,72 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>29,88 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>53,72 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>86,90 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>53,72 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Subtotal:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TENCIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ubtotal:</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added sum but features of delete total is disapeared
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="10">
   <si>
     <t>Concepto</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>Ref Reserva: 32373942 (26/05/2026 - 01/06/2026)</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
@@ -50,8 +53,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -79,9 +90,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -376,7 +388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
@@ -401,7 +413,7 @@
         <v>53.72</v>
       </c>
       <c r="C2" s="1">
-        <v>109.15</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -460,632 +472,349 @@
       </c>
     </row>
     <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>53.72</v>
+      </c>
       <c r="C8" s="1">
-        <v>0</v>
+        <v>109.15</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B9">
         <v>53.72</v>
       </c>
       <c r="C9" s="1">
-        <v>109.15</v>
+        <v>87.73</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10">
         <v>53.72</v>
       </c>
       <c r="C10" s="1">
-        <v>87.73</v>
+        <v>37.64</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B11">
         <v>53.72</v>
       </c>
       <c r="C11" s="1">
-        <v>37.64</v>
+        <v>85.91</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B12">
         <v>53.72</v>
       </c>
       <c r="C12" s="1">
-        <v>85.91</v>
+        <v>29.88</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13">
         <v>53.72</v>
       </c>
       <c r="C13" s="1">
-        <v>29.88</v>
+        <v>86.90000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B14">
         <v>53.72</v>
       </c>
       <c r="C14" s="1">
-        <v>86.90000000000001</v>
+        <v>109.15</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>53.72</v>
       </c>
       <c r="C15" s="1">
-        <v>109.15</v>
+        <v>87.73</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B16">
         <v>53.72</v>
       </c>
       <c r="C16" s="1">
-        <v>87.73</v>
+        <v>37.64</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B17">
         <v>53.72</v>
       </c>
       <c r="C17" s="1">
-        <v>37.64</v>
+        <v>85.91</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B18">
         <v>53.72</v>
       </c>
       <c r="C18" s="1">
-        <v>85.91</v>
+        <v>29.88</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B19">
         <v>53.72</v>
       </c>
       <c r="C19" s="1">
-        <v>29.88</v>
+        <v>86.90000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B20">
         <v>53.72</v>
       </c>
       <c r="C20" s="1">
-        <v>86.90000000000001</v>
+        <v>109.15</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B21">
         <v>53.72</v>
       </c>
       <c r="C21" s="1">
-        <v>109.15</v>
+        <v>87.73</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B22">
         <v>53.72</v>
       </c>
       <c r="C22" s="1">
-        <v>87.73</v>
+        <v>37.64</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B23">
         <v>53.72</v>
       </c>
       <c r="C23" s="1">
-        <v>37.64</v>
+        <v>85.91</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B24">
         <v>53.72</v>
       </c>
       <c r="C24" s="1">
-        <v>85.91</v>
+        <v>29.88</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B25">
         <v>53.72</v>
       </c>
       <c r="C25" s="1">
-        <v>29.88</v>
+        <v>86.90000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B26">
         <v>53.72</v>
       </c>
       <c r="C26" s="1">
-        <v>86.90000000000001</v>
+        <v>109.15</v>
       </c>
     </row>
     <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B27">
+        <v>53.72</v>
+      </c>
       <c r="C27" s="1">
-        <v>0</v>
+        <v>87.73</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B28">
         <v>53.72</v>
       </c>
       <c r="C28" s="1">
-        <v>109.15</v>
+        <v>37.64</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B29">
         <v>53.72</v>
       </c>
       <c r="C29" s="1">
-        <v>87.73</v>
+        <v>85.91</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B30">
         <v>53.72</v>
       </c>
       <c r="C30" s="1">
-        <v>37.64</v>
+        <v>29.88</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B31">
         <v>53.72</v>
       </c>
       <c r="C31" s="1">
-        <v>85.91</v>
+        <v>86.90000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32">
-        <v>53.72</v>
+      <c r="B32" t="s">
+        <v>9</v>
       </c>
       <c r="C32" s="1">
-        <v>29.88</v>
+        <v>2298.9</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B33">
         <v>53.72</v>
       </c>
       <c r="C33" s="1">
-        <v>86.90000000000001</v>
+        <v>109.15</v>
       </c>
     </row>
     <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34">
+        <v>53.72</v>
+      </c>
       <c r="C34" s="1">
-        <v>0</v>
+        <v>87.73</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B35">
         <v>53.72</v>
       </c>
       <c r="C35" s="1">
-        <v>2</v>
+        <v>37.64</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B36">
         <v>53.72</v>
       </c>
       <c r="C36" s="1">
-        <v>3</v>
+        <v>85.91</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B37">
         <v>53.72</v>
       </c>
       <c r="C37" s="1">
-        <v>37.64</v>
+        <v>29.88</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B38">
         <v>53.72</v>
       </c>
       <c r="C38" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>7</v>
-      </c>
-      <c r="B39">
-        <v>53.72</v>
-      </c>
-      <c r="C39" s="1">
-        <v>29.88</v>
+        <v>86.90000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>8</v>
-      </c>
-      <c r="B40">
-        <v>53.72</v>
+      <c r="B40" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="C40" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="C41" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>3</v>
-      </c>
-      <c r="B42">
-        <v>53.72</v>
-      </c>
-      <c r="C42" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>4</v>
-      </c>
-      <c r="B43">
-        <v>53.72</v>
-      </c>
-      <c r="C43" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>5</v>
-      </c>
-      <c r="B44">
-        <v>53.72</v>
-      </c>
-      <c r="C44" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>6</v>
-      </c>
-      <c r="B45">
-        <v>53.72</v>
-      </c>
-      <c r="C45" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" t="s">
-        <v>7</v>
-      </c>
-      <c r="B46">
-        <v>53.72</v>
-      </c>
-      <c r="C46" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" t="s">
-        <v>8</v>
-      </c>
-      <c r="B47">
-        <v>53.72</v>
-      </c>
-      <c r="C47" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="C48" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" t="s">
-        <v>3</v>
-      </c>
-      <c r="B49">
-        <v>53.72</v>
-      </c>
-      <c r="C49" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" t="s">
-        <v>4</v>
-      </c>
-      <c r="B50">
-        <v>53.72</v>
-      </c>
-      <c r="C50" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51" t="s">
-        <v>5</v>
-      </c>
-      <c r="B51">
-        <v>53.72</v>
-      </c>
-      <c r="C51" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
-        <v>6</v>
-      </c>
-      <c r="B52">
-        <v>53.72</v>
-      </c>
-      <c r="C52" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
-        <v>7</v>
-      </c>
-      <c r="B53">
-        <v>53.72</v>
-      </c>
-      <c r="C53" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" t="s">
-        <v>8</v>
-      </c>
-      <c r="B54">
-        <v>53.72</v>
-      </c>
-      <c r="C54" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="C55" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" t="s">
-        <v>3</v>
-      </c>
-      <c r="B56">
-        <v>53.72</v>
-      </c>
-      <c r="C56" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" t="s">
-        <v>4</v>
-      </c>
-      <c r="B57">
-        <v>53.72</v>
-      </c>
-      <c r="C57" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" t="s">
-        <v>5</v>
-      </c>
-      <c r="B58">
-        <v>53.72</v>
-      </c>
-      <c r="C58" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59" t="s">
-        <v>6</v>
-      </c>
-      <c r="B59">
-        <v>53.72</v>
-      </c>
-      <c r="C59" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60" t="s">
-        <v>7</v>
-      </c>
-      <c r="B60">
-        <v>53.72</v>
-      </c>
-      <c r="C60" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61" t="s">
-        <v>8</v>
-      </c>
-      <c r="B61">
-        <v>53.72</v>
-      </c>
-      <c r="C61" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="C62" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" t="s">
-        <v>3</v>
-      </c>
-      <c r="B63">
-        <v>53.72</v>
-      </c>
-      <c r="C63" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64" t="s">
-        <v>4</v>
-      </c>
-      <c r="B64">
-        <v>53.72</v>
-      </c>
-      <c r="C64" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" t="s">
-        <v>5</v>
-      </c>
-      <c r="B65">
-        <v>53.72</v>
-      </c>
-      <c r="C65" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" t="s">
-        <v>6</v>
-      </c>
-      <c r="B66">
-        <v>53.72</v>
-      </c>
-      <c r="C66" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" t="s">
-        <v>7</v>
-      </c>
-      <c r="B67">
-        <v>53.72</v>
-      </c>
-      <c r="C67" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" t="s">
-        <v>8</v>
-      </c>
-      <c r="B68">
-        <v>53.72</v>
-      </c>
-      <c r="C68" s="1">
-        <f>SUM(C2:C67)</f>
+        <f>SUM(C2:C38)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Import Error: The Panda don't read the input dataframe, but it solved by AI. And it's solved to the total rewrite
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
   <si>
     <t>Concepto</t>
   </si>
@@ -388,7 +388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
@@ -413,7 +413,7 @@
         <v>53.72</v>
       </c>
       <c r="C2" s="1">
-        <v>222</v>
+        <v>109.15</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -538,283 +538,11 @@
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14">
-        <v>53.72</v>
+      <c r="B14" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="C14" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15">
-        <v>53.72</v>
-      </c>
-      <c r="C15" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16">
-        <v>53.72</v>
-      </c>
-      <c r="C16" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17">
-        <v>53.72</v>
-      </c>
-      <c r="C17" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18">
-        <v>53.72</v>
-      </c>
-      <c r="C18" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19">
-        <v>53.72</v>
-      </c>
-      <c r="C19" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20">
-        <v>53.72</v>
-      </c>
-      <c r="C20" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21">
-        <v>53.72</v>
-      </c>
-      <c r="C21" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22">
-        <v>53.72</v>
-      </c>
-      <c r="C22" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23">
-        <v>53.72</v>
-      </c>
-      <c r="C23" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24">
-        <v>53.72</v>
-      </c>
-      <c r="C24" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>8</v>
-      </c>
-      <c r="B25">
-        <v>53.72</v>
-      </c>
-      <c r="C25" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26">
-        <v>53.72</v>
-      </c>
-      <c r="C26" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B27">
-        <v>53.72</v>
-      </c>
-      <c r="C27" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
-        <v>5</v>
-      </c>
-      <c r="B28">
-        <v>53.72</v>
-      </c>
-      <c r="C28" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29">
-        <v>53.72</v>
-      </c>
-      <c r="C29" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30">
-        <v>53.72</v>
-      </c>
-      <c r="C30" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31">
-        <v>53.72</v>
-      </c>
-      <c r="C31" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="B32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" s="1">
-        <v>2298.9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33">
-        <v>53.72</v>
-      </c>
-      <c r="C33" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>4</v>
-      </c>
-      <c r="B34">
-        <v>53.72</v>
-      </c>
-      <c r="C34" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>5</v>
-      </c>
-      <c r="B35">
-        <v>53.72</v>
-      </c>
-      <c r="C35" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>6</v>
-      </c>
-      <c r="B36">
-        <v>53.72</v>
-      </c>
-      <c r="C36" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37">
-        <v>53.72</v>
-      </c>
-      <c r="C37" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" t="s">
-        <v>8</v>
-      </c>
-      <c r="B38">
-        <v>53.72</v>
-      </c>
-      <c r="C38" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="B40" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" s="1">
-        <f>SUM(C2:C38)</f>
+        <f>SUM(C2:C1000)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
solved error of Err:512, expand the limits to one more row down to avoid recalling sum, because sum have to be outside of their own range and not be within
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="10">
   <si>
     <t>Concepto</t>
   </si>
@@ -388,7 +388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
@@ -413,7 +413,7 @@
         <v>53.72</v>
       </c>
       <c r="C2" s="1">
-        <v>109.15</v>
+        <v>1029.15</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -538,11 +538,77 @@
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="B14" s="2" t="s">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <v>53.72</v>
+      </c>
+      <c r="C14" s="1">
+        <v>109.15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15">
+        <v>53.72</v>
+      </c>
+      <c r="C15" s="1">
+        <v>87.73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>53.72</v>
+      </c>
+      <c r="C16" s="1">
+        <v>37.64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17">
+        <v>53.72</v>
+      </c>
+      <c r="C17" s="1">
+        <v>85.91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18">
+        <v>53.72</v>
+      </c>
+      <c r="C18" s="1">
+        <v>29.88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19">
+        <v>53.72</v>
+      </c>
+      <c r="C19" s="1">
+        <v>86.90000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="B21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="1">
-        <f>SUM(C2:C1000)</f>
+      <c r="C21" s="1">
+        <f>SUM(C2:C19)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Calculation of dates: there is an misundesrtanding about the rest of dates
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="10">
   <si>
     <t>Concepto</t>
   </si>
@@ -388,7 +388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
@@ -413,7 +413,7 @@
         <v>53.72</v>
       </c>
       <c r="C2" s="1">
-        <v>1029.15</v>
+        <v>109.15</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -603,12 +603,86 @@
         <v>86.90000000000001</v>
       </c>
     </row>
+    <row r="20" spans="1:3">
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1311.63</v>
+      </c>
+    </row>
     <row r="21" spans="1:3">
-      <c r="B21" s="2" t="s">
+      <c r="A21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21">
+        <v>53.72</v>
+      </c>
+      <c r="C21" s="1">
+        <v>109.15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22">
+        <v>53.72</v>
+      </c>
+      <c r="C22" s="1">
+        <v>87.73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23">
+        <v>53.72</v>
+      </c>
+      <c r="C23" s="1">
+        <v>37.64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24">
+        <v>53.72</v>
+      </c>
+      <c r="C24" s="1">
+        <v>85.91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25">
+        <v>53.72</v>
+      </c>
+      <c r="C25" s="1">
+        <v>29.88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26">
+        <v>53.72</v>
+      </c>
+      <c r="C26" s="1">
+        <v>86.90000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="B28" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="1">
-        <f>SUM(C2:C19)</f>
+      <c r="C28" s="1">
+        <f>SUM(C2:C26)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added calculation of dates
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -14,9 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Concepto</t>
+  </si>
+  <si>
+    <t>Noches</t>
   </si>
   <si>
     <t>Limpieza</t>
@@ -388,13 +391,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="15.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -404,285 +407,100 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1">
         <v>53.72</v>
       </c>
-      <c r="C2" s="1">
+      <c r="D2">
         <v>109.15</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
         <v>4</v>
       </c>
-      <c r="B3">
+      <c r="C3" s="1">
         <v>53.72</v>
       </c>
-      <c r="C3" s="1">
+      <c r="D3">
         <v>87.73</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D4">
+        <v>37.64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D5">
+        <v>85.91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D6">
+        <v>29.88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
         <v>5</v>
       </c>
-      <c r="B4">
+      <c r="C7" s="1">
         <v>53.72</v>
       </c>
-      <c r="C4" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>53.72</v>
-      </c>
-      <c r="C5" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6">
-        <v>53.72</v>
-      </c>
-      <c r="C6" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>53.72</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="D7">
         <v>86.90000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8">
-        <v>53.72</v>
-      </c>
-      <c r="C8" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9">
-        <v>53.72</v>
+    <row r="9" spans="1:4">
+      <c r="B9" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="C9" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10">
-        <v>53.72</v>
-      </c>
-      <c r="C10" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11">
-        <v>53.72</v>
-      </c>
-      <c r="C11" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12">
-        <v>53.72</v>
-      </c>
-      <c r="C12" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13">
-        <v>53.72</v>
-      </c>
-      <c r="C13" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14">
-        <v>53.72</v>
-      </c>
-      <c r="C14" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15">
-        <v>53.72</v>
-      </c>
-      <c r="C15" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16">
-        <v>53.72</v>
-      </c>
-      <c r="C16" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17">
-        <v>53.72</v>
-      </c>
-      <c r="C17" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18">
-        <v>53.72</v>
-      </c>
-      <c r="C18" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19">
-        <v>53.72</v>
-      </c>
-      <c r="C19" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="B20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="1">
-        <v>1311.63</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21">
-        <v>53.72</v>
-      </c>
-      <c r="C21" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22">
-        <v>53.72</v>
-      </c>
-      <c r="C22" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23">
-        <v>53.72</v>
-      </c>
-      <c r="C23" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24">
-        <v>53.72</v>
-      </c>
-      <c r="C24" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25">
-        <v>53.72</v>
-      </c>
-      <c r="C25" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>8</v>
-      </c>
-      <c r="B26">
-        <v>53.72</v>
-      </c>
-      <c r="C26" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="B28" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" s="1">
-        <f>SUM(C2:C26)</f>
+        <f>SUM(C2:C7)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
The totals doesn't appear twice
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
   <si>
     <t>Concepto</t>
   </si>
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="4" width="15.7109375" style="1" customWidth="1"/>
@@ -507,60 +507,144 @@
         <v>86.90000000000001</v>
       </c>
     </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D8" s="1">
+        <v>109.15</v>
+      </c>
+    </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D9" s="1">
+        <v>87.73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D10" s="1">
+        <v>37.64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D11" s="1">
+        <v>85.91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D12" s="1">
+        <v>29.88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <v>5</v>
+      </c>
+      <c r="C13" s="1">
+        <v>53.72</v>
+      </c>
+      <c r="D13" s="1">
+        <v>86.90000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9">
-        <f>SUM(B2:B7)</f>
-        <v>0</v>
-      </c>
-      <c r="C9" s="1">
-        <f>SUM(C2:C7)</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="1">
-        <f>SUM(D2:D7)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="2" t="s">
+      <c r="B15">
+        <f>SUM(B2:B13)</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="1">
+        <f>SUM(C2:C13)</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
+        <f>SUM(D2:D13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="1">
-        <f>SUM(C9)*0.21</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="1">
-        <f>SUM(D9)*0.21</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="2" t="s">
+      <c r="C16" s="1">
+        <f>SUM(C15)*0.21</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
+        <f>SUM(D15)*0.21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="1">
-        <f>SUM(C10, D10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="2" t="s">
+      <c r="D17" s="1">
+        <f>SUM(C16, D16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="1">
-        <f>SUM(C9,D9)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="2" t="s">
+      <c r="D18" s="1">
+        <f>SUM(C15,D15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="1">
-        <f>SUM(D11, D12)</f>
+      <c r="D19" s="1">
+        <f>SUM(D17, D18)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add selected multiples files
</commit_message>
<xml_diff>
--- a/resumen_facturas.xlsx
+++ b/resumen_facturas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Concepto</t>
   </si>
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="4" width="15.7109375" style="1" customWidth="1"/>
@@ -508,311 +508,67 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
       <c r="B8">
-        <v>6</v>
-      </c>
-      <c r="C8" s="1">
-        <v>53.72</v>
+        <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9">
-        <v>4</v>
-      </c>
-      <c r="C9" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D9" s="1">
-        <v>87.73</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>6</v>
+      <c r="A10" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <f>SUM(B2:B8)</f>
+        <v>0</v>
       </c>
       <c r="C10" s="1">
-        <v>53.72</v>
+        <f>SUM(C2:C8)</f>
+        <v>0</v>
       </c>
       <c r="D10" s="1">
-        <v>37.64</v>
+        <f>SUM(D2:D8)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11">
-        <v>4</v>
+      <c r="A11" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="C11" s="1">
-        <v>53.72</v>
+        <f>SUM(C10)*0.21</f>
+        <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>85.91</v>
+        <f>SUM(D10)*0.21</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12">
-        <v>1</v>
-      </c>
-      <c r="C12" s="1">
-        <v>53.72</v>
+      <c r="A12" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="D12" s="1">
-        <v>29.88</v>
+        <f>SUM(C11, D11)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13">
-        <v>5</v>
-      </c>
-      <c r="C13" s="1">
-        <v>53.72</v>
+      <c r="A13" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="D13" s="1">
-        <v>86.90000000000001</v>
+        <f>SUM(C10,D10)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14">
-        <v>6</v>
-      </c>
-      <c r="C14" s="1">
-        <v>53.72</v>
+      <c r="A14" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="D14" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15">
-        <v>4</v>
-      </c>
-      <c r="C15" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D15" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>6</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D16" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17">
-        <v>4</v>
-      </c>
-      <c r="C17" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D17" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D18" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19">
-        <v>5</v>
-      </c>
-      <c r="C19" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D19" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20">
-        <v>6</v>
-      </c>
-      <c r="C20" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D20" s="1">
-        <v>109.15</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21">
-        <v>4</v>
-      </c>
-      <c r="C21" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D21" s="1">
-        <v>87.73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
-        <v>6</v>
-      </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-      <c r="C22" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D22" s="1">
-        <v>37.64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23">
-        <v>4</v>
-      </c>
-      <c r="C23" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D23" s="1">
-        <v>85.91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-      <c r="C24" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D24" s="1">
-        <v>29.88</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25">
-        <v>5</v>
-      </c>
-      <c r="C25" s="1">
-        <v>53.72</v>
-      </c>
-      <c r="D25" s="1">
-        <v>86.90000000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27">
-        <f>SUM(B2:B25)</f>
-        <v>0</v>
-      </c>
-      <c r="C27" s="1">
-        <f>SUM(C2:C25)</f>
-        <v>0</v>
-      </c>
-      <c r="D27" s="1">
-        <f>SUM(D2:D25)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" s="1">
-        <f>SUM(C27)*0.21</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="1">
-        <f>SUM(D27)*0.21</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="1">
-        <f>SUM(C28, D28)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" s="1">
-        <f>SUM(C27,D27)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D31" s="1">
-        <f>SUM(D29, D30)</f>
+        <f>SUM(D12, D13)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>